<commit_message>
[IMP] stock: improve the import function of detail stock overview
The template for inventory adjustments was a generic template.
This makes it hard for the user to actually use the template for a stock adjustment.
To improve the UX the template is now preloaded with all the stockable products.
This template can be used to set the new values.
The column Inventory Quantity and Product Name is indicative for the user.

Task-6164275
</commit_message>
<xml_diff>
--- a/addons/stock/static/xlsx/stock_quant.xlsx
+++ b/addons/stock/static/xlsx/stock_quant.xlsx
@@ -1,94 +1,93 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr defaultThemeVersion="124226"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr fullCalcOnLoad="1"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>Product</t>
   </si>
   <si>
-    <t>Lot/Serial Number</t>
+    <t xml:space="preserve">Lot/Serial Number</t>
   </si>
   <si>
     <t>Quantity</t>
   </si>
   <si>
-    <t>Counted Quantity</t>
-  </si>
-  <si>
-    <t>Difference</t>
-  </si>
-  <si>
-    <t>Scheduled Date</t>
-  </si>
-  <si>
-    <t>Assigned To</t>
-  </si>
-  <si>
-    <t>[FURN_0789] Individual Workplace</t>
-  </si>
-  <si>
-    <t>[E-COM08] Storage Box</t>
-  </si>
-  <si>
-    <t>[E-COM07] Large Cabinet</t>
-  </si>
-  <si>
-    <t>[E-COM10] Pedal Bin</t>
-  </si>
-  <si>
-    <t>[E-COM11] Cabinet with Doors</t>
-  </si>
-  <si>
-    <t>[E-COM12] Conference Chair (Steel)</t>
-  </si>
-  <si>
-    <t>[E-COM13] Conference Chair (Aluminium)</t>
-  </si>
-  <si>
-    <t>[FURN_0096] Customizable Desk (Steel, White)</t>
-  </si>
-  <si>
-    <t>[FURN_0097] Customizable Desk (Steel, Black)</t>
-  </si>
-  <si>
-    <t>[FURN_0098] Customizable Desk (Aluminium, White)</t>
-  </si>
-  <si>
-    <t>[DESK0004] Customizable Desk (Aluminium, Black)</t>
-  </si>
-  <si>
-    <t>[FURN_0269] Office Chair Black</t>
-  </si>
-  <si>
-    <t>[FURN_1118] Corner Desk Left Sit</t>
-  </si>
-  <si>
-    <t>[FURN_8855] Drawer</t>
+    <t xml:space="preserve">Counted Quantity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scheduled Date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assigned To</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[FURN_0789] Individual Workplace</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[E-COM08] Storage Box</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[E-COM07] Large Cabinet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[E-COM10] Pedal Bin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[E-COM11] Cabinet with Doors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[E-COM12] Conference Chair (Steel)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[E-COM13] Conference Chair (Aluminium)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[FURN_0096] Customizable Desk (Steel, White)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[FURN_0097] Customizable Desk (Steel, Black)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[FURN_0098] Customizable Desk (Aluminium, White)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[DESK0004] Customizable Desk (Aluminium, Black)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[FURN_0269] Office Chair Black</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[FURN_1118] Corner Desk Left Sit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[FURN_8855] Drawer</t>
   </si>
   <si>
     <t>0000000000029</t>
   </si>
   <si>
-    <t>[FURN_7800] Desk Combination</t>
-  </si>
-  <si>
-    <t>[FURN_6666] Acoustic Bloc Screens</t>
-  </si>
-  <si>
-    <t>[FURN_5555] Cable Management Box</t>
+    <t xml:space="preserve">[FURN_7800] Desk Combination</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[FURN_6666] Acoustic Bloc Screens</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[FURN_5555] Cable Management Box</t>
   </si>
   <si>
     <t>CM-BOX-00001</t>
@@ -100,24 +99,22 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="2">
     <font>
-      <sz val="11"/>
+      <sz val="11.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="11.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -131,23 +128,23 @@
   </fills>
   <borders count="1">
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
   <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -155,11 +152,16 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/theme/theme.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -205,13 +207,13 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Jpan" typeface="ＭＳ ゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
         <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Thai" typeface="Angsana New"/>
         <a:font script="Ethi" typeface="Nyala"/>
         <a:font script="Beng" typeface="Vrinda"/>
         <a:font script="Gujr" typeface="Shruti"/>
@@ -239,13 +241,13 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Jpan" typeface="ＭＳ 明朝"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
         <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Thai" typeface="Cordia New"/>
         <a:font script="Ethi" typeface="Nyala"/>
         <a:font script="Beng" typeface="Vrinda"/>
         <a:font script="Gujr" typeface="Shruti"/>
@@ -442,15 +444,234 @@
 </a:theme>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface="Arial"/>
+        <a:cs typeface="Arial"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface="Arial"/>
+        <a:cs typeface="Arial"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle"/>
+        </a:gradFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G19"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="7" width="30.7109375" customWidth="1"/>
+    <col customWidth="1" min="1" max="7" width="30.7109375"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -469,13 +690,10 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="s">
         <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" s="2" t="s">
-        <v>7</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2">
@@ -484,17 +702,14 @@
       <c r="D2" s="2">
         <v>0</v>
       </c>
-      <c r="E2" s="2">
-        <v>0</v>
-      </c>
-      <c r="F2" s="3">
-        <v>44926</v>
-      </c>
-      <c r="G2" s="2"/>
-    </row>
-    <row r="3" spans="1:7">
+      <c r="E2" s="3">
+        <v>44926</v>
+      </c>
+      <c r="F2" s="2"/>
+    </row>
+    <row r="3">
       <c r="A3" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2">
@@ -503,17 +718,14 @@
       <c r="D3" s="2">
         <v>0</v>
       </c>
-      <c r="E3" s="2">
-        <v>0</v>
-      </c>
-      <c r="F3" s="3">
-        <v>44926</v>
-      </c>
-      <c r="G3" s="2"/>
-    </row>
-    <row r="4" spans="1:7">
+      <c r="E3" s="3">
+        <v>44926</v>
+      </c>
+      <c r="F3" s="2"/>
+    </row>
+    <row r="4">
       <c r="A4" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2">
@@ -522,17 +734,14 @@
       <c r="D4" s="2">
         <v>0</v>
       </c>
-      <c r="E4" s="2">
-        <v>0</v>
-      </c>
-      <c r="F4" s="3">
-        <v>44926</v>
-      </c>
-      <c r="G4" s="2"/>
-    </row>
-    <row r="5" spans="1:7">
+      <c r="E4" s="3">
+        <v>44926</v>
+      </c>
+      <c r="F4" s="2"/>
+    </row>
+    <row r="5">
       <c r="A5" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2">
@@ -541,17 +750,14 @@
       <c r="D5" s="2">
         <v>0</v>
       </c>
-      <c r="E5" s="2">
-        <v>0</v>
-      </c>
-      <c r="F5" s="3">
-        <v>44926</v>
-      </c>
-      <c r="G5" s="2"/>
-    </row>
-    <row r="6" spans="1:7">
+      <c r="E5" s="3">
+        <v>44926</v>
+      </c>
+      <c r="F5" s="2"/>
+    </row>
+    <row r="6">
       <c r="A6" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2">
@@ -560,17 +766,14 @@
       <c r="D6" s="2">
         <v>0</v>
       </c>
-      <c r="E6" s="2">
-        <v>0</v>
-      </c>
-      <c r="F6" s="3">
-        <v>44926</v>
-      </c>
-      <c r="G6" s="2"/>
-    </row>
-    <row r="7" spans="1:7">
+      <c r="E6" s="3">
+        <v>44926</v>
+      </c>
+      <c r="F6" s="2"/>
+    </row>
+    <row r="7">
       <c r="A7" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="2">
@@ -579,17 +782,14 @@
       <c r="D7" s="2">
         <v>0</v>
       </c>
-      <c r="E7" s="2">
-        <v>0</v>
-      </c>
-      <c r="F7" s="3">
-        <v>44926</v>
-      </c>
-      <c r="G7" s="2"/>
-    </row>
-    <row r="8" spans="1:7">
+      <c r="E7" s="3">
+        <v>44926</v>
+      </c>
+      <c r="F7" s="2"/>
+    </row>
+    <row r="8" ht="28.5">
       <c r="A8" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2">
@@ -598,17 +798,14 @@
       <c r="D8" s="2">
         <v>0</v>
       </c>
-      <c r="E8" s="2">
-        <v>0</v>
-      </c>
-      <c r="F8" s="3">
-        <v>44926</v>
-      </c>
-      <c r="G8" s="2"/>
-    </row>
-    <row r="9" spans="1:7">
+      <c r="E8" s="3">
+        <v>44926</v>
+      </c>
+      <c r="F8" s="2"/>
+    </row>
+    <row r="9" ht="28.5">
       <c r="A9" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" s="2">
@@ -617,17 +814,14 @@
       <c r="D9" s="2">
         <v>0</v>
       </c>
-      <c r="E9" s="2">
-        <v>0</v>
-      </c>
-      <c r="F9" s="3">
-        <v>44926</v>
-      </c>
-      <c r="G9" s="2"/>
-    </row>
-    <row r="10" spans="1:7">
+      <c r="E9" s="3">
+        <v>44926</v>
+      </c>
+      <c r="F9" s="2"/>
+    </row>
+    <row r="10" ht="28.5">
       <c r="A10" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2">
@@ -636,17 +830,14 @@
       <c r="D10" s="2">
         <v>0</v>
       </c>
-      <c r="E10" s="2">
-        <v>0</v>
-      </c>
-      <c r="F10" s="3">
-        <v>44926</v>
-      </c>
-      <c r="G10" s="2"/>
-    </row>
-    <row r="11" spans="1:7">
+      <c r="E10" s="3">
+        <v>44926</v>
+      </c>
+      <c r="F10" s="2"/>
+    </row>
+    <row r="11" ht="28.5">
       <c r="A11" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" s="2">
@@ -655,17 +846,14 @@
       <c r="D11" s="2">
         <v>0</v>
       </c>
-      <c r="E11" s="2">
-        <v>0</v>
-      </c>
-      <c r="F11" s="3">
-        <v>44926</v>
-      </c>
-      <c r="G11" s="2"/>
-    </row>
-    <row r="12" spans="1:7">
+      <c r="E11" s="3">
+        <v>44926</v>
+      </c>
+      <c r="F11" s="2"/>
+    </row>
+    <row r="12" ht="28.5">
       <c r="A12" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" s="2">
@@ -674,17 +862,14 @@
       <c r="D12" s="2">
         <v>0</v>
       </c>
-      <c r="E12" s="2">
-        <v>0</v>
-      </c>
-      <c r="F12" s="3">
-        <v>44926</v>
-      </c>
-      <c r="G12" s="2"/>
-    </row>
-    <row r="13" spans="1:7">
+      <c r="E12" s="3">
+        <v>44926</v>
+      </c>
+      <c r="F12" s="2"/>
+    </row>
+    <row r="13">
       <c r="A13" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="2">
@@ -693,17 +878,14 @@
       <c r="D13" s="2">
         <v>0</v>
       </c>
-      <c r="E13" s="2">
-        <v>0</v>
-      </c>
-      <c r="F13" s="3">
-        <v>44926</v>
-      </c>
-      <c r="G13" s="2"/>
-    </row>
-    <row r="14" spans="1:7">
+      <c r="E13" s="3">
+        <v>44926</v>
+      </c>
+      <c r="F13" s="2"/>
+    </row>
+    <row r="14">
       <c r="A14" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="2">
@@ -712,20 +894,17 @@
       <c r="D14" s="2">
         <v>0</v>
       </c>
-      <c r="E14" s="2">
-        <v>0</v>
-      </c>
-      <c r="F14" s="3">
-        <v>44926</v>
-      </c>
-      <c r="G14" s="2"/>
-    </row>
-    <row r="15" spans="1:7">
+      <c r="E14" s="3">
+        <v>44926</v>
+      </c>
+      <c r="F14" s="2"/>
+    </row>
+    <row r="15">
       <c r="A15" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>20</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>21</v>
       </c>
       <c r="C15" s="2">
         <v>80</v>
@@ -733,17 +912,14 @@
       <c r="D15" s="2">
         <v>0</v>
       </c>
-      <c r="E15" s="2">
-        <v>0</v>
-      </c>
-      <c r="F15" s="3">
-        <v>44926</v>
-      </c>
-      <c r="G15" s="2"/>
-    </row>
-    <row r="16" spans="1:7">
+      <c r="E15" s="3">
+        <v>44926</v>
+      </c>
+      <c r="F15" s="2"/>
+    </row>
+    <row r="16">
       <c r="A16" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="2">
@@ -752,17 +928,14 @@
       <c r="D16" s="2">
         <v>0</v>
       </c>
-      <c r="E16" s="2">
-        <v>0</v>
-      </c>
-      <c r="F16" s="3">
-        <v>44926</v>
-      </c>
-      <c r="G16" s="2"/>
-    </row>
-    <row r="17" spans="1:7">
+      <c r="E16" s="3">
+        <v>44926</v>
+      </c>
+      <c r="F16" s="2"/>
+    </row>
+    <row r="17">
       <c r="A17" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B17" s="2"/>
       <c r="C17" s="2">
@@ -771,20 +944,17 @@
       <c r="D17" s="2">
         <v>0</v>
       </c>
-      <c r="E17" s="2">
-        <v>0</v>
-      </c>
-      <c r="F17" s="3">
-        <v>44926</v>
-      </c>
-      <c r="G17" s="2"/>
-    </row>
-    <row r="18" spans="1:7">
+      <c r="E17" s="3">
+        <v>44926</v>
+      </c>
+      <c r="F17" s="2"/>
+    </row>
+    <row r="18" ht="28.5">
       <c r="A18" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B18" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>25</v>
       </c>
       <c r="C18" s="2">
         <v>50</v>
@@ -792,20 +962,17 @@
       <c r="D18" s="2">
         <v>0</v>
       </c>
-      <c r="E18" s="2">
-        <v>0</v>
-      </c>
-      <c r="F18" s="3">
-        <v>44926</v>
-      </c>
-      <c r="G18" s="2"/>
-    </row>
-    <row r="19" spans="1:7">
+      <c r="E18" s="3">
+        <v>44926</v>
+      </c>
+      <c r="F18" s="2"/>
+    </row>
+    <row r="19" ht="28.5">
       <c r="A19" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C19" s="2">
         <v>40</v>
@@ -813,15 +980,15 @@
       <c r="D19" s="2">
         <v>0</v>
       </c>
-      <c r="E19" s="2">
-        <v>0</v>
-      </c>
-      <c r="F19" s="3">
-        <v>44926</v>
-      </c>
-      <c r="G19" s="2"/>
+      <c r="E19" s="3">
+        <v>44926</v>
+      </c>
+      <c r="F19" s="2"/>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>